<commit_message>
Completar matriz RACI con reparto de roles por componente
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantilla/mcu5/excel/03-matriz-raci-mcu5.xlsx
+++ b/plantilla/mcu5/excel/03-matriz-raci-mcu5.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz RACI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matriz RACI" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,261 +493,261 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Gestión de incidentes</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Analista/SOC</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Dueños de activos, TI</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Procedimiento de incidentes</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Registros de incidentes</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gestion de incidentes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Andres Varela (deteccion via SIEM/dashboard)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Horacio Duarte y Pablo Morales (duenos del componente afectado)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Todo el equipo (bitacora)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>docs/04-Gestion-Incidentes.md (pendiente)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Registro de incidentes en control-central + docs/evidencias</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Gestión de accesos</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Admin IAM</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Jefes de unidad</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Dueños de activos</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Política de accesos</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Matriz de accesos y revisión</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gestion de accesos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Horacio Duarte (MFA local, cliente-gestor); Pablo Morales (RBAC/hash, control-central)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>El otro dueno de componente en cada caso</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>docs/09-Gestion-Accesos.md</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Capturas de enroll TOTP/WebAuthn/Hello + config del hash (pendientes de implementacion)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Evaluación de riesgos</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Dueños de procesos</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Auditoría</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Metodología ISO 31000</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Matriz de riesgos</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Evaluacion de riesgos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Andres Varela</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Horacio Duarte y Pablo Morales (detalle tecnico por componente)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>docs/03-Analisis-Riesgos.md</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Matriz de riesgos (12 riesgos, R01-R12)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Gestión de vulnerabilidades</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Equipo TI</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Dueños de activos</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Procedimiento de parcheo</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Registro con CVSS/SLA</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gestion de vulnerabilidades</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Horacio Duarte (cliente-gestor); Pablo Morales (control-central/infra)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>docs/10-Gestion-Vulnerabilidades.md (pendiente)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Escaneos SAST/DAST/OpenVAS (pendientes)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Capacitación</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>RRHH + RSI</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Jefaturas</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Plan anual</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Registro de asistencia</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Capacitacion / induccion del equipo</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Andres Varela (coordinacion)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Horacio Duarte y Pablo Morales</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>docs/01-Politica-Seguridad.md, docs/99-bitacora-trabajo.md</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Entradas de bitacora de repaso de la letra</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Continuidad (BCP/DRP)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Tecnología</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Jefaturas</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>BIA + BCP</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Prueba de restauración</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pablo Morales (infra: backups control-central/Wazuh/Mailu); Horacio Duarte (export/import de bovedas)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>docs/06-Plan-Continuidad.md (pendiente)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Prueba de restauracion (pendiente)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Notificación a autoridades</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>RSI</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Procedimiento de notificación</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Borradores + constancias</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Notificacion a autoridades (BCU/URCDP)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Andres Varela (RSI)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Horacio Duarte y Pablo Morales (detalle tecnico del incidente)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>docs/12-Notificacion-Incidentes.md (pendiente)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Borradores de notificacion simulada</t>
         </is>
       </c>
     </row>

</xml_diff>